<commit_message>
correction of compare with duckdb + small corrections
</commit_message>
<xml_diff>
--- a/tests-assets/Budget2025_Asia.xlsx
+++ b/tests-assets/Budget2025_Asia.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qnsv2207\Documents\tests_alteryx_tableau_qlik\pour_amphi\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qnsv2207\amphi_dev\fix-compare-duckdb\amphi-etl\tests-assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41716DA2-7BE9-4EB8-80AC-AC727E79BDFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78EE9F57-9887-4F01-B5A7-194BD2B6B86D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -798,9 +798,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter>
-    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Helvetica 75 Bold"&amp;8&amp;KED7D31 Orange Restricted</oddFooter>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -1161,9 +1158,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter>
-    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Helvetica 75 Bold"&amp;8&amp;KED7D31 Orange Restricted</oddFooter>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -1524,14 +1518,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter>
-    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Helvetica 75 Bold"&amp;8&amp;KED7D31 Orange Restricted</oddFooter>
-  </headerFooter>
 </worksheet>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{e6c818a6-e1a0-4a6e-a969-20d857c5dc62}" enabled="1" method="Standard" siteId="{90c7a20a-f34b-40bf-bc48-b9253b6f5d20}" contentBits="2" removed="0"/>
+  <clbl:label id="{07222825-62ea-40f3-96b5-5375c07996e2}" enabled="1" method="Privileged" siteId="{90c7a20a-f34b-40bf-bc48-b9253b6f5d20}" contentBits="0" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>